<commit_message>
fix(viewer): Import's dialog: steps' buttons, Cancel, beside Export
</commit_message>
<xml_diff>
--- a/demos/samples/contacts-to-import.xlsx
+++ b/demos/samples/contacts-to-import.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
     <t>Full name</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Customer</t>
   </si>
   <si>
-    <t>Mona Adel</t>
+    <t>Sara Haddad</t>
   </si>
   <si>
     <t>Orders every month</t>
@@ -90,91 +90,94 @@
     <t>Lead</t>
   </si>
   <si>
+    <t>Lina Khalil</t>
+  </si>
+  <si>
+    <t>Leila Mansour</t>
+  </si>
+  <si>
+    <t>Petra Tours</t>
+  </si>
+  <si>
+    <t>leila.mansour@petratours.example</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>Faisal Al-Harbi</t>
+  </si>
+  <si>
+    <t>Red Sea Divers</t>
+  </si>
+  <si>
+    <t>faisal.alharbi@redseadivers.example</t>
+  </si>
+  <si>
+    <t>Saudi Arabia</t>
+  </si>
+  <si>
+    <t>Prefers WhatsApp</t>
+  </si>
+  <si>
+    <t>Hannah Becker</t>
+  </si>
+  <si>
+    <t>Cedar Logistics</t>
+  </si>
+  <si>
+    <t>hannah.becker@cedarlogistics.example</t>
+  </si>
+  <si>
+    <t>Lucas Moreau</t>
+  </si>
+  <si>
+    <t>Atlas Builders</t>
+  </si>
+  <si>
+    <t>lucas.moreau@atlasbuilders.example</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>Karim Nasser</t>
+  </si>
+  <si>
+    <t>Priya Raman</t>
+  </si>
+  <si>
+    <t>Lotus Spa</t>
+  </si>
+  <si>
+    <t>priya.raman@lotusspa.example</t>
+  </si>
+  <si>
+    <t>Met at the Riyadh fair</t>
+  </si>
+  <si>
+    <t>Kenji Watanabe</t>
+  </si>
+  <si>
+    <t>Harbour Freight</t>
+  </si>
+  <si>
+    <t>kenji.watanabe@harbourfreight.example</t>
+  </si>
+  <si>
+    <t>Sofia Rossi</t>
+  </si>
+  <si>
+    <t>Saffron Kitchens</t>
+  </si>
+  <si>
+    <t>sofia.rossi@saffronkitchens.example</t>
+  </si>
+  <si>
     <t>Omar Said</t>
   </si>
   <si>
-    <t>Leila Mansour</t>
-  </si>
-  <si>
-    <t>Petra Tours</t>
-  </si>
-  <si>
-    <t>leila.mansour@petratours.example</t>
-  </si>
-  <si>
-    <t>Jordan</t>
-  </si>
-  <si>
-    <t>Sara Haddad</t>
-  </si>
-  <si>
-    <t>Faisal Al-Harbi</t>
-  </si>
-  <si>
-    <t>Red Sea Divers</t>
-  </si>
-  <si>
-    <t>faisal.alharbi@redseadivers.example</t>
-  </si>
-  <si>
-    <t>Saudi Arabia</t>
-  </si>
-  <si>
-    <t>Lina Khalil</t>
-  </si>
-  <si>
-    <t>Prefers WhatsApp</t>
-  </si>
-  <si>
-    <t>Hannah Becker</t>
-  </si>
-  <si>
-    <t>Cedar Logistics</t>
-  </si>
-  <si>
-    <t>hannah.becker@cedarlogistics.example</t>
-  </si>
-  <si>
-    <t>Lucas Moreau</t>
-  </si>
-  <si>
-    <t>Atlas Builders</t>
-  </si>
-  <si>
-    <t>lucas.moreau@atlasbuilders.example</t>
-  </si>
-  <si>
-    <t>Inactive</t>
-  </si>
-  <si>
-    <t>Priya Raman</t>
-  </si>
-  <si>
-    <t>Lotus Spa</t>
-  </si>
-  <si>
-    <t>priya.raman@lotusspa.example</t>
-  </si>
-  <si>
-    <t>Met at the Riyadh fair</t>
-  </si>
-  <si>
-    <t>Kenji Watanabe</t>
-  </si>
-  <si>
-    <t>Harbour Freight</t>
-  </si>
-  <si>
-    <t>kenji.watanabe@harbourfreight.example</t>
-  </si>
-  <si>
-    <t>Sofia Rossi</t>
-  </si>
-  <si>
-    <t>Saffron Kitchens</t>
-  </si>
-  <si>
-    <t>sofia.rossi@saffronkitchens.example</t>
+    <t>Two users are called Omar Said</t>
   </si>
   <si>
     <t>Oasis Water</t>
@@ -421,7 +424,7 @@
         <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G4" s="1">
         <v>46205</v>
@@ -432,22 +435,22 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>29</v>
       </c>
       <c r="E5" t="s">
         <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G5" s="1">
         <v>46162</v>
@@ -456,18 +459,18 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
         <v>32</v>
-      </c>
-      <c r="B6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -484,22 +487,22 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
         <v>35</v>
-      </c>
-      <c r="B7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="G7" s="1">
         <v>45964</v>
@@ -510,39 +513,39 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
         <v>39</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>40</v>
       </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
         <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s">
         <v>43</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>44</v>
-      </c>
-      <c r="C9" t="s">
-        <v>45</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
@@ -551,7 +554,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G9" s="1">
         <v>46263</v>
@@ -562,13 +565,13 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
         <v>46</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>47</v>
-      </c>
-      <c r="C11" t="s">
-        <v>48</v>
       </c>
       <c r="D11" t="s">
         <v>24</v>
@@ -577,7 +580,7 @@
         <v>13</v>
       </c>
       <c r="F11" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G11" s="1">
         <v>46184</v>
@@ -585,13 +588,16 @@
       <c r="H11" t="b">
         <v>1</v>
       </c>
+      <c r="I11" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="12" spans="1:9">
       <c r="B12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -600,33 +606,33 @@
         <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>
@@ -634,22 +640,22 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
         <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H14" t="b">
         <v>0</v>
@@ -657,13 +663,13 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -672,7 +678,7 @@
         <v>13</v>
       </c>
       <c r="F15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G15" s="1">
         <v>46130</v>
@@ -683,13 +689,13 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D16" t="s">
         <v>24</v>
@@ -698,27 +704,27 @@
         <v>13</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H16" t="b">
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
@@ -727,30 +733,30 @@
         <v>19</v>
       </c>
       <c r="F17" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="H17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E18" t="s">
         <v>13</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G18" s="1">
         <v>46088</v>
@@ -761,13 +767,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>

</xml_diff>